<commit_message>
Stage 8 review fixes: D-013
</commit_message>
<xml_diff>
--- a/output/archive/Archive/Users/cstrachan_old_laptop/commercial/2022/compchem-scope-rates-v3 (2).xlsx
+++ b/output/archive/Archive/Users/cstrachan_old_laptop/commercial/2022/compchem-scope-rates-v3 (2).xlsx
@@ -166,12 +166,12 @@
   <commentList>
     <comment ref="C3" authorId="0" shapeId="0">
       <text>
-        <t>Dataset rate assumes the standard reanalysis pipeline. Custom pipelines are a new scope.</t>
+        <t>Confirm the RNA-seq analysis steps and input data in the engagement scope; custom pipeline work needs an explicit scope before quoting.</t>
       </text>
     </comment>
     <comment ref="E3" authorId="1" shapeId="0">
       <text>
-        <t>Callum: 'none' is what we have actually been applying, but the old note mentioned a volume discount. Needs checking with finance before the rates go out.</t>
+        <t>Callum: the list has no automatic volume discount. Record any proposed negotiated discount separately on the engagement sheet and obtain approval before issue.</t>
       </text>
     </comment>
   </commentList>
@@ -683,7 +683,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Note: docking and hit clustering are scoped as part of virtual library triage and not priced separately in this sheet.</t>
+          <t>Note: docking and hit clustering have no separate list rate on this sheet. Confirm their inclusion and scope in the engagement quote.</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Typical scope</t>
+          <t>Proposed scope for discussion</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Full library screen with docking and clustering</t>
+          <t>Library triage; confirm whether docking and clustering are requested</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -808,6 +808,18 @@
       <c r="C6" s="2" t="inlineStr">
         <is>
           <t>RNA-seq differential expression</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Effort bands are scoping prompts, not price multipliers or guaranteed inclusions. Confirm the biological question, input provenance and analysis steps in each quote.</t>
         </is>
       </c>
     </row>

</xml_diff>